<commit_message>
iOS Honeycomb: move steal-mode instruction into the rules pill
The floating "Double-tap a captured opponent's card..." banner + Cancel button
covered the board cards it was telling the player to tap. Steal mode now
borrows the always-visible rules pill instead (topBar in landscape, rulesCapsule
in portrait), with shorter text ("Double-tap to steal a card") that fits one
line. No cancel button: Rematch/Start already exit steal mode via the
gameState-leaves-.gameOver reset added earlier.

Adds steal_instruction_tap_compact to the localization spreadsheet and
regenerates every platform's generated string tables.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F707"/>
+  <dimension ref="A1:F708"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20175,27 +20175,27 @@
     <row r="655">
       <c r="A655" t="inlineStr">
         <is>
-          <t>TouchViewsIOS</t>
+          <t>Honeycomb</t>
         </is>
       </c>
       <c r="B655" t="inlineStr">
         <is>
-          <t>touch_layout_coming_soon</t>
+          <t>steal_instruction_tap_compact</t>
         </is>
       </c>
       <c r="C655" t="inlineStr">
         <is>
-          <t>Placeholder/fallback text</t>
+          <t>Steal-mode instructional hint shown in the compact top-bar rules pill (replaces the rule name while steal mode is active) — short enough to fit that one-line pill instead of steal_instruction_tap's full two-line wording.</t>
         </is>
       </c>
       <c r="D655" t="inlineStr">
         <is>
-          <t>Touch layout coming soon</t>
+          <t>Double-tap to steal a card</t>
         </is>
       </c>
       <c r="E655" t="inlineStr">
         <is>
-          <t>Diseño táctil próximamente</t>
+          <t>Toca dos veces para robar una carta</t>
         </is>
       </c>
       <c r="F655" t="b">
@@ -20210,26 +20210,26 @@
       </c>
       <c r="B656" t="inlineStr">
         <is>
-          <t>touch_blackjack_title</t>
+          <t>touch_layout_coming_soon</t>
         </is>
       </c>
       <c r="C656" t="inlineStr">
         <is>
-          <t>Title-case game label</t>
+          <t>Placeholder/fallback text</t>
         </is>
       </c>
       <c r="D656" t="inlineStr">
         <is>
-          <t>Blackjack</t>
+          <t>Touch layout coming soon</t>
         </is>
       </c>
       <c r="E656" t="inlineStr">
         <is>
-          <t>Blackjack</t>
+          <t>Diseño táctil próximamente</t>
         </is>
       </c>
       <c r="F656" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="657">
@@ -20240,22 +20240,22 @@
       </c>
       <c r="B657" t="inlineStr">
         <is>
-          <t>touch_blackjack_banner</t>
+          <t>touch_blackjack_title</t>
         </is>
       </c>
       <c r="C657" t="inlineStr">
         <is>
-          <t>All-caps banner/header label</t>
+          <t>Title-case game label</t>
         </is>
       </c>
       <c r="D657" t="inlineStr">
         <is>
-          <t>BLACKJACK</t>
+          <t>Blackjack</t>
         </is>
       </c>
       <c r="E657" t="inlineStr">
         <is>
-          <t>BLACKJACK</t>
+          <t>Blackjack</t>
         </is>
       </c>
       <c r="F657" t="b">
@@ -20270,7 +20270,7 @@
       </c>
       <c r="B658" t="inlineStr">
         <is>
-          <t>touch_spider_banner</t>
+          <t>touch_blackjack_banner</t>
         </is>
       </c>
       <c r="C658" t="inlineStr">
@@ -20280,12 +20280,12 @@
       </c>
       <c r="D658" t="inlineStr">
         <is>
-          <t>SPIDER</t>
+          <t>BLACKJACK</t>
         </is>
       </c>
       <c r="E658" t="inlineStr">
         <is>
-          <t>SPIDER</t>
+          <t>BLACKJACK</t>
         </is>
       </c>
       <c r="F658" t="b">
@@ -20300,7 +20300,7 @@
       </c>
       <c r="B659" t="inlineStr">
         <is>
-          <t>touch_klondike_banner</t>
+          <t>touch_spider_banner</t>
         </is>
       </c>
       <c r="C659" t="inlineStr">
@@ -20310,12 +20310,12 @@
       </c>
       <c r="D659" t="inlineStr">
         <is>
-          <t>KLONDIKE</t>
+          <t>SPIDER</t>
         </is>
       </c>
       <c r="E659" t="inlineStr">
         <is>
-          <t>KLONDIKE</t>
+          <t>SPIDER</t>
         </is>
       </c>
       <c r="F659" t="b">
@@ -20330,7 +20330,7 @@
       </c>
       <c r="B660" t="inlineStr">
         <is>
-          <t>touch_beecell_banner</t>
+          <t>touch_klondike_banner</t>
         </is>
       </c>
       <c r="C660" t="inlineStr">
@@ -20340,12 +20340,12 @@
       </c>
       <c r="D660" t="inlineStr">
         <is>
-          <t>BEECELL</t>
+          <t>KLONDIKE</t>
         </is>
       </c>
       <c r="E660" t="inlineStr">
         <is>
-          <t>BEECELL</t>
+          <t>KLONDIKE</t>
         </is>
       </c>
       <c r="F660" t="b">
@@ -20355,57 +20355,57 @@
     <row r="661">
       <c r="A661" t="inlineStr">
         <is>
-          <t>Chrome</t>
+          <t>TouchViewsIOS</t>
         </is>
       </c>
       <c r="B661" t="inlineStr">
         <is>
-          <t>debug_banners_menu</t>
+          <t>touch_beecell_banner</t>
         </is>
       </c>
       <c r="C661" t="inlineStr">
         <is>
-          <t>Mac-only dev menu title</t>
+          <t>All-caps banner/header label</t>
         </is>
       </c>
       <c r="D661" t="inlineStr">
         <is>
-          <t>Banners</t>
+          <t>BEECELL</t>
         </is>
       </c>
       <c r="E661" t="inlineStr">
         <is>
-          <t>Anuncios</t>
+          <t>BEECELL</t>
         </is>
       </c>
       <c r="F661" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="662">
       <c r="A662" t="inlineStr">
         <is>
-          <t>ManageDecksWin</t>
+          <t>Chrome</t>
         </is>
       </c>
       <c r="B662" t="inlineStr">
         <is>
-          <t>deck_default_name</t>
+          <t>debug_banners_menu</t>
         </is>
       </c>
       <c r="C662" t="inlineStr">
         <is>
-          <t>Windows Manage Decks: display name for the slot-0 (default) deck</t>
+          <t>Mac-only dev menu title</t>
         </is>
       </c>
       <c r="D662" t="inlineStr">
         <is>
-          <t>Default</t>
+          <t>Banners</t>
         </is>
       </c>
       <c r="E662" t="inlineStr">
         <is>
-          <t>Predeterminado</t>
+          <t>Anuncios</t>
         </is>
       </c>
       <c r="F662" t="b">
@@ -20415,27 +20415,27 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>TouchViewsIOS</t>
+          <t>ManageDecksWin</t>
         </is>
       </c>
       <c r="B663" t="inlineStr">
         <is>
-          <t>free_play_label</t>
+          <t>deck_default_name</t>
         </is>
       </c>
       <c r="C663" t="inlineStr">
         <is>
-          <t>iOS Blackjack/Video Poker touch view: credits capsule label in free-play mode</t>
+          <t>Windows Manage Decks: display name for the slot-0 (default) deck</t>
         </is>
       </c>
       <c r="D663" t="inlineStr">
         <is>
-          <t>Free Play</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="E663" t="inlineStr">
         <is>
-          <t>Juego Libre</t>
+          <t>Predeterminado</t>
         </is>
       </c>
       <c r="F663" t="b">
@@ -20450,22 +20450,22 @@
       </c>
       <c r="B664" t="inlineStr">
         <is>
-          <t>touch_choose_photo</t>
+          <t>free_play_label</t>
         </is>
       </c>
       <c r="C664" t="inlineStr">
         <is>
-          <t>iOS custom-art import sheets: photo picker button, no image chosen yet</t>
+          <t>iOS Blackjack/Video Poker touch view: credits capsule label in free-play mode</t>
         </is>
       </c>
       <c r="D664" t="inlineStr">
         <is>
-          <t>Choose Photo</t>
+          <t>Free Play</t>
         </is>
       </c>
       <c r="E664" t="inlineStr">
         <is>
-          <t>Elegir Foto</t>
+          <t>Juego Libre</t>
         </is>
       </c>
       <c r="F664" t="b">
@@ -20480,22 +20480,22 @@
       </c>
       <c r="B665" t="inlineStr">
         <is>
-          <t>touch_choose_different_photo</t>
+          <t>touch_choose_photo</t>
         </is>
       </c>
       <c r="C665" t="inlineStr">
         <is>
-          <t>iOS custom-art import sheets: photo picker button, image already chosen</t>
+          <t>iOS custom-art import sheets: photo picker button, no image chosen yet</t>
         </is>
       </c>
       <c r="D665" t="inlineStr">
         <is>
-          <t>Choose a Different Photo</t>
+          <t>Choose Photo</t>
         </is>
       </c>
       <c r="E665" t="inlineStr">
         <is>
-          <t>Elegir Otra Foto</t>
+          <t>Elegir Foto</t>
         </is>
       </c>
       <c r="F665" t="b">
@@ -20510,22 +20510,22 @@
       </c>
       <c r="B666" t="inlineStr">
         <is>
-          <t>touch_pinch_zoom_reposition</t>
+          <t>touch_choose_different_photo</t>
         </is>
       </c>
       <c r="C666" t="inlineStr">
         <is>
-          <t>iOS custom-art import sheets: crop editor section header</t>
+          <t>iOS custom-art import sheets: photo picker button, image already chosen</t>
         </is>
       </c>
       <c r="D666" t="inlineStr">
         <is>
-          <t>Pinch to zoom, drag to reposition</t>
+          <t>Choose a Different Photo</t>
         </is>
       </c>
       <c r="E666" t="inlineStr">
         <is>
-          <t>Pellizca para hacer zoom, arrastra para reposicionar</t>
+          <t>Elegir Otra Foto</t>
         </is>
       </c>
       <c r="F666" t="b">
@@ -20540,22 +20540,22 @@
       </c>
       <c r="B667" t="inlineStr">
         <is>
-          <t>touch_name_field_placeholder</t>
+          <t>touch_pinch_zoom_reposition</t>
         </is>
       </c>
       <c r="C667" t="inlineStr">
         <is>
-          <t>iOS custom-art import sheets: name TextField placeholder</t>
+          <t>iOS custom-art import sheets: crop editor section header</t>
         </is>
       </c>
       <c r="D667" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Pinch to zoom, drag to reposition</t>
         </is>
       </c>
       <c r="E667" t="inlineStr">
         <is>
-          <t>Nombre</t>
+          <t>Pellizca para hacer zoom, arrastra para reposicionar</t>
         </is>
       </c>
       <c r="F667" t="b">
@@ -20570,22 +20570,22 @@
       </c>
       <c r="B668" t="inlineStr">
         <is>
-          <t>touch_name_already_taken_error</t>
+          <t>touch_name_field_placeholder</t>
         </is>
       </c>
       <c r="C668" t="inlineStr">
         <is>
-          <t>iOS custom-art import sheets: duplicate-name validation error</t>
+          <t>iOS custom-art import sheets: name TextField placeholder</t>
         </is>
       </c>
       <c r="D668" t="inlineStr">
         <is>
-          <t>That name is already taken — pick another.</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="E668" t="inlineStr">
         <is>
-          <t>Ese nombre ya está en uso — elige otro.</t>
+          <t>Nombre</t>
         </is>
       </c>
       <c r="F668" t="b">
@@ -20600,22 +20600,22 @@
       </c>
       <c r="B669" t="inlineStr">
         <is>
-          <t>touch_enabled_toggle</t>
+          <t>touch_name_already_taken_error</t>
         </is>
       </c>
       <c r="C669" t="inlineStr">
         <is>
-          <t>iOS custom face-card-art import sheet: Enabled toggle label</t>
+          <t>iOS custom-art import sheets: duplicate-name validation error</t>
         </is>
       </c>
       <c r="D669" t="inlineStr">
         <is>
-          <t>Enabled</t>
+          <t>That name is already taken — pick another.</t>
         </is>
       </c>
       <c r="E669" t="inlineStr">
         <is>
-          <t>Activado</t>
+          <t>Ese nombre ya está en uso — elige otro.</t>
         </is>
       </c>
       <c r="F669" t="b">
@@ -20630,22 +20630,22 @@
       </c>
       <c r="B670" t="inlineStr">
         <is>
-          <t>card_back_default_name</t>
+          <t>touch_enabled_toggle</t>
         </is>
       </c>
       <c r="C670" t="inlineStr">
         <is>
-          <t>Auto-filled base name for a new custom card back before the user renames it (appended with ' N' for the 2nd, 3rd, ... duplicate)</t>
+          <t>iOS custom face-card-art import sheet: Enabled toggle label</t>
         </is>
       </c>
       <c r="D670" t="inlineStr">
         <is>
-          <t>Default</t>
+          <t>Enabled</t>
         </is>
       </c>
       <c r="E670" t="inlineStr">
         <is>
-          <t>Predeterminado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="F670" t="b">
@@ -20660,22 +20660,22 @@
       </c>
       <c r="B671" t="inlineStr">
         <is>
-          <t>add_photo_short</t>
+          <t>card_back_default_name</t>
         </is>
       </c>
       <c r="C671" t="inlineStr">
         <is>
-          <t>Caption on the iOS Themes sheet Background grid's Add tile (imports a photo, unlike Card Back/Face Art's plain "Add")</t>
+          <t>Auto-filled base name for a new custom card back before the user renames it (appended with ' N' for the 2nd, 3rd, ... duplicate)</t>
         </is>
       </c>
       <c r="D671" t="inlineStr">
         <is>
-          <t>Add Photo</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="E671" t="inlineStr">
         <is>
-          <t>Añadir Foto</t>
+          <t>Predeterminado</t>
         </is>
       </c>
       <c r="F671" t="b">
@@ -20690,22 +20690,22 @@
       </c>
       <c r="B672" t="inlineStr">
         <is>
-          <t>felt_custom_short</t>
+          <t>add_photo_short</t>
         </is>
       </c>
       <c r="C672" t="inlineStr">
         <is>
-          <t>Caption on the iOS Themes sheet Background grid's Custom Felt tile — shorter than feltCustomColor ("Custom Felt Color") so it fits the narrow tile without truncating</t>
+          <t>Caption on the iOS Themes sheet Background grid's Add tile (imports a photo, unlike Card Back/Face Art's plain "Add")</t>
         </is>
       </c>
       <c r="D672" t="inlineStr">
         <is>
-          <t>Custom Felt</t>
+          <t>Add Photo</t>
         </is>
       </c>
       <c r="E672" t="inlineStr">
         <is>
-          <t>Fieltro Personalizado</t>
+          <t>Añadir Foto</t>
         </is>
       </c>
       <c r="F672" t="b">
@@ -20720,22 +20720,22 @@
       </c>
       <c r="B673" t="inlineStr">
         <is>
-          <t>stat_position_top</t>
+          <t>felt_custom_short</t>
         </is>
       </c>
       <c r="C673" t="inlineStr">
         <is>
-          <t>Label on the iOS Card Bank stat-filter dropdown for a card's top corner value</t>
+          <t>Caption on the iOS Themes sheet Background grid's Custom Felt tile — shorter than feltCustomColor ("Custom Felt Color") so it fits the narrow tile without truncating</t>
         </is>
       </c>
       <c r="D673" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Custom Felt</t>
         </is>
       </c>
       <c r="E673" t="inlineStr">
         <is>
-          <t>Arriba</t>
+          <t>Fieltro Personalizado</t>
         </is>
       </c>
       <c r="F673" t="b">
@@ -20750,22 +20750,22 @@
       </c>
       <c r="B674" t="inlineStr">
         <is>
-          <t>stat_position_bottom</t>
+          <t>stat_position_top</t>
         </is>
       </c>
       <c r="C674" t="inlineStr">
         <is>
-          <t>Label on the iOS Card Bank stat-filter dropdown for a card's bottom corner value</t>
+          <t>Label on the iOS Card Bank stat-filter dropdown for a card's top corner value</t>
         </is>
       </c>
       <c r="D674" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="E674" t="inlineStr">
         <is>
-          <t>Abajo</t>
+          <t>Arriba</t>
         </is>
       </c>
       <c r="F674" t="b">
@@ -20780,22 +20780,22 @@
       </c>
       <c r="B675" t="inlineStr">
         <is>
-          <t>stat_position_left</t>
+          <t>stat_position_bottom</t>
         </is>
       </c>
       <c r="C675" t="inlineStr">
         <is>
-          <t>Label on the iOS Card Bank stat-filter dropdown for a card's left corner value</t>
+          <t>Label on the iOS Card Bank stat-filter dropdown for a card's bottom corner value</t>
         </is>
       </c>
       <c r="D675" t="inlineStr">
         <is>
-          <t>Left</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="E675" t="inlineStr">
         <is>
-          <t>Izquierda</t>
+          <t>Abajo</t>
         </is>
       </c>
       <c r="F675" t="b">
@@ -20810,22 +20810,22 @@
       </c>
       <c r="B676" t="inlineStr">
         <is>
-          <t>stat_position_right</t>
+          <t>stat_position_left</t>
         </is>
       </c>
       <c r="C676" t="inlineStr">
         <is>
-          <t>Label on the iOS Card Bank stat-filter dropdown for a card's right corner value</t>
+          <t>Label on the iOS Card Bank stat-filter dropdown for a card's left corner value</t>
         </is>
       </c>
       <c r="D676" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>Left</t>
         </is>
       </c>
       <c r="E676" t="inlineStr">
         <is>
-          <t>Derecha</t>
+          <t>Izquierda</t>
         </is>
       </c>
       <c r="F676" t="b">
@@ -20840,22 +20840,22 @@
       </c>
       <c r="B677" t="inlineStr">
         <is>
-          <t>stat_filter_any</t>
+          <t>stat_position_right</t>
         </is>
       </c>
       <c r="C677" t="inlineStr">
         <is>
-          <t>Default/unset option in each iOS Card Bank stat-filter dropdown (matches any value)</t>
+          <t>Label on the iOS Card Bank stat-filter dropdown for a card's right corner value</t>
         </is>
       </c>
       <c r="D677" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Right</t>
         </is>
       </c>
       <c r="E677" t="inlineStr">
         <is>
-          <t>Cualquiera</t>
+          <t>Derecha</t>
         </is>
       </c>
       <c r="F677" t="b">
@@ -20870,22 +20870,22 @@
       </c>
       <c r="B678" t="inlineStr">
         <is>
-          <t>stat_sudden_death_count_ios</t>
+          <t>stat_filter_any</t>
         </is>
       </c>
       <c r="C678" t="inlineStr">
         <is>
-          <t>iOS Honeycomb stats sheet label for suddenDeathCount — plainer than mac's thematic "Most Swarms to the Death", matching iOS's literal stat-label style</t>
+          <t>Default/unset option in each iOS Card Bank stat-filter dropdown (matches any value)</t>
         </is>
       </c>
       <c r="D678" t="inlineStr">
         <is>
-          <t>Most Swarms to the Death</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="E678" t="inlineStr">
         <is>
-          <t>Más Enjambres a Muerte</t>
+          <t>Cualquiera</t>
         </is>
       </c>
       <c r="F678" t="b">
@@ -20900,22 +20900,22 @@
       </c>
       <c r="B679" t="inlineStr">
         <is>
-          <t>stat_fallen_aces_ios</t>
+          <t>stat_sudden_death_count_ios</t>
         </is>
       </c>
       <c r="C679" t="inlineStr">
         <is>
-          <t>iOS Honeycomb stats sheet label for fallenAces — plainer than mac's thematic "Queen's Falls", matching iOS's literal stat-label style</t>
+          <t>iOS Honeycomb stats sheet label for suddenDeathCount — plainer than mac's thematic "Most Swarms to the Death", matching iOS's literal stat-label style</t>
         </is>
       </c>
       <c r="D679" t="inlineStr">
         <is>
-          <t>Queen's Falls</t>
+          <t>Most Swarms to the Death</t>
         </is>
       </c>
       <c r="E679" t="inlineStr">
         <is>
-          <t>Caídas de la Reina</t>
+          <t>Más Enjambres a Muerte</t>
         </is>
       </c>
       <c r="F679" t="b">
@@ -20925,27 +20925,27 @@
     <row r="680">
       <c r="A680" t="inlineStr">
         <is>
-          <t>Honeycomb</t>
+          <t>TouchViewsIOS</t>
         </is>
       </c>
       <c r="B680" t="inlineStr">
         <is>
-          <t>rule_state_auto</t>
+          <t>stat_fallen_aces_ios</t>
         </is>
       </c>
       <c r="C680" t="inlineStr">
         <is>
-          <t>Unified rule-list per-row state control, Mac/iOS/Windows</t>
+          <t>iOS Honeycomb stats sheet label for fallenAces — plainer than mac's thematic "Queen's Falls", matching iOS's literal stat-label style</t>
         </is>
       </c>
       <c r="D680" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Queen's Falls</t>
         </is>
       </c>
       <c r="E680" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Caídas de la Reina</t>
         </is>
       </c>
       <c r="F680" t="b">
@@ -20960,7 +20960,7 @@
       </c>
       <c r="B681" t="inlineStr">
         <is>
-          <t>rule_state_pick</t>
+          <t>rule_state_auto</t>
         </is>
       </c>
       <c r="C681" t="inlineStr">
@@ -20970,12 +20970,12 @@
       </c>
       <c r="D681" t="inlineStr">
         <is>
-          <t>Play</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="E681" t="inlineStr">
         <is>
-          <t>Jugar</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="F681" t="b">
@@ -20990,7 +20990,7 @@
       </c>
       <c r="B682" t="inlineStr">
         <is>
-          <t>rule_state_ban</t>
+          <t>rule_state_pick</t>
         </is>
       </c>
       <c r="C682" t="inlineStr">
@@ -21000,12 +21000,12 @@
       </c>
       <c r="D682" t="inlineStr">
         <is>
-          <t>Ban</t>
+          <t>Play</t>
         </is>
       </c>
       <c r="E682" t="inlineStr">
         <is>
-          <t>Vetar</t>
+          <t>Jugar</t>
         </is>
       </c>
       <c r="F682" t="b">
@@ -21020,22 +21020,22 @@
       </c>
       <c r="B683" t="inlineStr">
         <is>
-          <t>rules_selected_count_fmt</t>
+          <t>rule_state_ban</t>
         </is>
       </c>
       <c r="C683" t="inlineStr">
         <is>
-          <t>Unified rule-list selection counter, Mac/iOS/Windows</t>
+          <t>Unified rule-list per-row state control, Mac/iOS/Windows</t>
         </is>
       </c>
       <c r="D683" t="inlineStr">
         <is>
-          <t>%d of 4 selected</t>
+          <t>Ban</t>
         </is>
       </c>
       <c r="E683" t="inlineStr">
         <is>
-          <t>%d de 4 seleccionadas</t>
+          <t>Vetar</t>
         </is>
       </c>
       <c r="F683" t="b">
@@ -21045,27 +21045,27 @@
     <row r="684">
       <c r="A684" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>Honeycomb</t>
         </is>
       </c>
       <c r="B684" t="inlineStr">
         <is>
-          <t>out_of_credits_toast</t>
+          <t>rules_selected_count_fmt</t>
         </is>
       </c>
       <c r="C684" t="inlineStr">
         <is>
-          <t>Toast shown when the player runs out of credits, reused Blackjack/Video Poker</t>
+          <t>Unified rule-list selection counter, Mac/iOS/Windows</t>
         </is>
       </c>
       <c r="D684" t="inlineStr">
         <is>
-          <t>Out of Credits!</t>
+          <t>%d of 4 selected</t>
         </is>
       </c>
       <c r="E684" t="inlineStr">
         <is>
-          <t>¡Sin créditos!</t>
+          <t>%d de 4 seleccionadas</t>
         </is>
       </c>
       <c r="F684" t="b">
@@ -21075,27 +21075,27 @@
     <row r="685">
       <c r="A685" t="inlineStr">
         <is>
-          <t>Blackjack</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="B685" t="inlineStr">
         <is>
-          <t>btn_clear_short</t>
+          <t>out_of_credits_toast</t>
         </is>
       </c>
       <c r="C685" t="inlineStr">
         <is>
-          <t>Short "Clear" label for Blackjack landscape betting grid (fits one line at that button width)</t>
+          <t>Toast shown when the player runs out of credits, reused Blackjack/Video Poker</t>
         </is>
       </c>
       <c r="D685" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Out of Credits!</t>
         </is>
       </c>
       <c r="E685" t="inlineStr">
         <is>
-          <t>Borrar</t>
+          <t>¡Sin créditos!</t>
         </is>
       </c>
       <c r="F685" t="b">
@@ -21105,27 +21105,27 @@
     <row r="686">
       <c r="A686" t="inlineStr">
         <is>
-          <t>Options</t>
+          <t>Blackjack</t>
         </is>
       </c>
       <c r="B686" t="inlineStr">
         <is>
-          <t>global_options_section</t>
+          <t>btn_clear_short</t>
         </is>
       </c>
       <c r="C686" t="inlineStr">
         <is>
-          <t>iOS Options sheet section header — groups Sound/No Stress Mode/Honey Mode/Hide Hint/Manually Dismiss Banners, separate from the per-game settings section below it</t>
+          <t>Short "Clear" label for Blackjack landscape betting grid (fits one line at that button width)</t>
         </is>
       </c>
       <c r="D686" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="E686" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Borrar</t>
         </is>
       </c>
       <c r="F686" t="b">
@@ -21135,27 +21135,27 @@
     <row r="687">
       <c r="A687" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>Options</t>
         </is>
       </c>
       <c r="B687" t="inlineStr">
         <is>
-          <t>hide_bee</t>
+          <t>global_options_section</t>
         </is>
       </c>
       <c r="C687" t="inlineStr">
         <is>
-          <t>Toggle label, reused across every game's Options on Mac/iOS/Windows</t>
+          <t>iOS Options sheet section header — groups Sound/No Stress Mode/Honey Mode/Hide Hint/Manually Dismiss Banners, separate from the per-game settings section below it</t>
         </is>
       </c>
       <c r="D687" t="inlineStr">
         <is>
-          <t>Hide the Bee</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="E687" t="inlineStr">
         <is>
-          <t>Ocultar la Abeja</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="F687" t="b">
@@ -21165,27 +21165,27 @@
     <row r="688">
       <c r="A688" t="inlineStr">
         <is>
-          <t>Options</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="B688" t="inlineStr">
         <is>
-          <t>honey_mode_tooltip</t>
+          <t>hide_bee</t>
         </is>
       </c>
       <c r="C688" t="inlineStr">
         <is>
-          <t>Tooltip for the Honey Mode toggle</t>
+          <t>Toggle label, reused across every game's Options on Mac/iOS/Windows</t>
         </is>
       </c>
       <c r="D688" t="inlineStr">
         <is>
-          <t>Enables banners and solitaire point animations.</t>
+          <t>Hide the Bee</t>
         </is>
       </c>
       <c r="E688" t="inlineStr">
         <is>
-          <t>Habilita los anuncios y las animaciones de puntos en los solitarios.</t>
+          <t>Ocultar la Abeja</t>
         </is>
       </c>
       <c r="F688" t="b">
@@ -21200,22 +21200,22 @@
       </c>
       <c r="B689" t="inlineStr">
         <is>
-          <t>no_stress_mode_tooltip</t>
+          <t>honey_mode_tooltip</t>
         </is>
       </c>
       <c r="C689" t="inlineStr">
         <is>
-          <t>Tooltip for the No Stress Mode toggle</t>
+          <t>Tooltip for the Honey Mode toggle</t>
         </is>
       </c>
       <c r="D689" t="inlineStr">
         <is>
-          <t>Pressure-free! No timers, no betting, and Honeycomb chooses your deck for you at random.</t>
+          <t>Enables banners and solitaire point animations.</t>
         </is>
       </c>
       <c r="E689" t="inlineStr">
         <is>
-          <t>¡Sin presión! Sin temporizadores, sin apuestas, y Honeycomb elige tu mazo al azar.</t>
+          <t>Habilita los anuncios y las animaciones de puntos en los solitarios.</t>
         </is>
       </c>
       <c r="F689" t="b">
@@ -21225,27 +21225,27 @@
     <row r="690">
       <c r="A690" t="inlineStr">
         <is>
-          <t>Honeycomb</t>
+          <t>Options</t>
         </is>
       </c>
       <c r="B690" t="inlineStr">
         <is>
-          <t>rank_nurse_bee</t>
+          <t>no_stress_mode_tooltip</t>
         </is>
       </c>
       <c r="C690" t="inlineStr">
         <is>
-          <t>Player rank, 10-19 cards collected</t>
+          <t>Tooltip for the No Stress Mode toggle</t>
         </is>
       </c>
       <c r="D690" t="inlineStr">
         <is>
-          <t>Nurse Bee</t>
+          <t>Pressure-free! No timers, no betting, and Honeycomb chooses your deck for you at random.</t>
         </is>
       </c>
       <c r="E690" t="inlineStr">
         <is>
-          <t>Abeja Nodriza</t>
+          <t>¡Sin presión! Sin temporizadores, sin apuestas, y Honeycomb elige tu mazo al azar.</t>
         </is>
       </c>
       <c r="F690" t="b">
@@ -21260,22 +21260,22 @@
       </c>
       <c r="B691" t="inlineStr">
         <is>
-          <t>rank_scout_bee</t>
+          <t>rank_nurse_bee</t>
         </is>
       </c>
       <c r="C691" t="inlineStr">
         <is>
-          <t>Player rank, 20-49 cards collected</t>
+          <t>Player rank, 10-19 cards collected</t>
         </is>
       </c>
       <c r="D691" t="inlineStr">
         <is>
-          <t>Scout Bee</t>
+          <t>Nurse Bee</t>
         </is>
       </c>
       <c r="E691" t="inlineStr">
         <is>
-          <t>Abeja Exploradora</t>
+          <t>Abeja Nodriza</t>
         </is>
       </c>
       <c r="F691" t="b">
@@ -21290,22 +21290,22 @@
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>rank_worker_bee</t>
+          <t>rank_scout_bee</t>
         </is>
       </c>
       <c r="C692" t="inlineStr">
         <is>
-          <t>Player rank, 50-99 cards collected</t>
+          <t>Player rank, 20-49 cards collected</t>
         </is>
       </c>
       <c r="D692" t="inlineStr">
         <is>
-          <t>Worker Bee</t>
+          <t>Scout Bee</t>
         </is>
       </c>
       <c r="E692" t="inlineStr">
         <is>
-          <t>Abeja Obrera</t>
+          <t>Abeja Exploradora</t>
         </is>
       </c>
       <c r="F692" t="b">
@@ -21320,22 +21320,22 @@
       </c>
       <c r="B693" t="inlineStr">
         <is>
-          <t>rank_guard_bee</t>
+          <t>rank_worker_bee</t>
         </is>
       </c>
       <c r="C693" t="inlineStr">
         <is>
-          <t>Player rank, 100-149 cards collected</t>
+          <t>Player rank, 50-99 cards collected</t>
         </is>
       </c>
       <c r="D693" t="inlineStr">
         <is>
-          <t>Guard Bee</t>
+          <t>Worker Bee</t>
         </is>
       </c>
       <c r="E693" t="inlineStr">
         <is>
-          <t>Abeja Guardiana</t>
+          <t>Abeja Obrera</t>
         </is>
       </c>
       <c r="F693" t="b">
@@ -21350,22 +21350,22 @@
       </c>
       <c r="B694" t="inlineStr">
         <is>
-          <t>rank_waggle_dancer</t>
+          <t>rank_guard_bee</t>
         </is>
       </c>
       <c r="C694" t="inlineStr">
         <is>
-          <t>Player rank, 150-199 cards collected</t>
+          <t>Player rank, 100-149 cards collected</t>
         </is>
       </c>
       <c r="D694" t="inlineStr">
         <is>
-          <t>Waggle Dancer</t>
+          <t>Guard Bee</t>
         </is>
       </c>
       <c r="E694" t="inlineStr">
         <is>
-          <t>Abeja Bailarina</t>
+          <t>Abeja Guardiana</t>
         </is>
       </c>
       <c r="F694" t="b">
@@ -21380,22 +21380,22 @@
       </c>
       <c r="B695" t="inlineStr">
         <is>
-          <t>rank_comb_architect</t>
+          <t>rank_waggle_dancer</t>
         </is>
       </c>
       <c r="C695" t="inlineStr">
         <is>
-          <t>Player rank, 200-299 cards collected</t>
+          <t>Player rank, 150-199 cards collected</t>
         </is>
       </c>
       <c r="D695" t="inlineStr">
         <is>
-          <t>Comb Architect</t>
+          <t>Waggle Dancer</t>
         </is>
       </c>
       <c r="E695" t="inlineStr">
         <is>
-          <t>Arquitecta del Panal</t>
+          <t>Abeja Bailarina</t>
         </is>
       </c>
       <c r="F695" t="b">
@@ -21410,22 +21410,22 @@
       </c>
       <c r="B696" t="inlineStr">
         <is>
-          <t>rank_royal_attendant</t>
+          <t>rank_comb_architect</t>
         </is>
       </c>
       <c r="C696" t="inlineStr">
         <is>
-          <t>Player rank, 300-399 cards collected</t>
+          <t>Player rank, 200-299 cards collected</t>
         </is>
       </c>
       <c r="D696" t="inlineStr">
         <is>
-          <t>Royal Attendant</t>
+          <t>Comb Architect</t>
         </is>
       </c>
       <c r="E696" t="inlineStr">
         <is>
-          <t>Asistente Real</t>
+          <t>Arquitecta del Panal</t>
         </is>
       </c>
       <c r="F696" t="b">
@@ -21440,22 +21440,22 @@
       </c>
       <c r="B697" t="inlineStr">
         <is>
-          <t>rank_swarm_leader</t>
+          <t>rank_royal_attendant</t>
         </is>
       </c>
       <c r="C697" t="inlineStr">
         <is>
-          <t>Player rank, 400-499 cards collected</t>
+          <t>Player rank, 300-399 cards collected</t>
         </is>
       </c>
       <c r="D697" t="inlineStr">
         <is>
-          <t>Swarm Leader</t>
+          <t>Royal Attendant</t>
         </is>
       </c>
       <c r="E697" t="inlineStr">
         <is>
-          <t>Líder del Enjambre</t>
+          <t>Asistente Real</t>
         </is>
       </c>
       <c r="F697" t="b">
@@ -21470,22 +21470,22 @@
       </c>
       <c r="B698" t="inlineStr">
         <is>
-          <t>rank_hive_monarch</t>
+          <t>rank_swarm_leader</t>
         </is>
       </c>
       <c r="C698" t="inlineStr">
         <is>
-          <t>Player rank, 500+ cards collected but not the full set</t>
+          <t>Player rank, 400-499 cards collected</t>
         </is>
       </c>
       <c r="D698" t="inlineStr">
         <is>
-          <t>Hive Monarch</t>
+          <t>Swarm Leader</t>
         </is>
       </c>
       <c r="E698" t="inlineStr">
         <is>
-          <t>Monarca de la Colmena</t>
+          <t>Líder del Enjambre</t>
         </is>
       </c>
       <c r="F698" t="b">
@@ -21500,22 +21500,22 @@
       </c>
       <c r="B699" t="inlineStr">
         <is>
-          <t>rank_apiarist</t>
+          <t>rank_hive_monarch</t>
         </is>
       </c>
       <c r="C699" t="inlineStr">
         <is>
-          <t>Player rank, every card in the collection unlocked</t>
+          <t>Player rank, 500+ cards collected but not the full set</t>
         </is>
       </c>
       <c r="D699" t="inlineStr">
         <is>
-          <t>Apiarist</t>
+          <t>Hive Monarch</t>
         </is>
       </c>
       <c r="E699" t="inlineStr">
         <is>
-          <t>Apicultor</t>
+          <t>Monarca de la Colmena</t>
         </is>
       </c>
       <c r="F699" t="b">
@@ -21525,27 +21525,27 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>Honeycomb</t>
         </is>
       </c>
       <c r="B700" t="inlineStr">
         <is>
-          <t>global_settings_header</t>
+          <t>rank_apiarist</t>
         </is>
       </c>
       <c r="C700" t="inlineStr">
         <is>
-          <t>Section header, Windows Preferences panel — global (cross-game) settings group</t>
+          <t>Player rank, every card in the collection unlocked</t>
         </is>
       </c>
       <c r="D700" t="inlineStr">
         <is>
-          <t>Global Settings</t>
+          <t>Apiarist</t>
         </is>
       </c>
       <c r="E700" t="inlineStr">
         <is>
-          <t>Configuración Global</t>
+          <t>Apicultor</t>
         </is>
       </c>
       <c r="F700" t="b">
@@ -21555,27 +21555,27 @@
     <row r="701">
       <c r="A701" t="inlineStr">
         <is>
-          <t>Stats</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="B701" t="inlineStr">
         <is>
-          <t>stat_shortest_win_time</t>
+          <t>global_settings_header</t>
         </is>
       </c>
       <c r="C701" t="inlineStr">
         <is>
-          <t>Stat row label, Klondike/Spider/Beecell — shortest winning-game time</t>
+          <t>Section header, Windows Preferences panel — global (cross-game) settings group</t>
         </is>
       </c>
       <c r="D701" t="inlineStr">
         <is>
-          <t>Shortest Win Time</t>
+          <t>Global Settings</t>
         </is>
       </c>
       <c r="E701" t="inlineStr">
         <is>
-          <t>Tiempo Más Corto de Victoria</t>
+          <t>Configuración Global</t>
         </is>
       </c>
       <c r="F701" t="b">
@@ -21590,22 +21590,22 @@
       </c>
       <c r="B702" t="inlineStr">
         <is>
-          <t>stat_total_paid_out</t>
+          <t>stat_shortest_win_time</t>
         </is>
       </c>
       <c r="C702" t="inlineStr">
         <is>
-          <t>Stat row label, Blackjack/Video Poker</t>
+          <t>Stat row label, Klondike/Spider/Beecell — shortest winning-game time</t>
         </is>
       </c>
       <c r="D702" t="inlineStr">
         <is>
-          <t>Total Paid Out</t>
+          <t>Shortest Win Time</t>
         </is>
       </c>
       <c r="E702" t="inlineStr">
         <is>
-          <t>Total Pagado</t>
+          <t>Tiempo Más Corto de Victoria</t>
         </is>
       </c>
       <c r="F702" t="b">
@@ -21620,7 +21620,7 @@
       </c>
       <c r="B703" t="inlineStr">
         <is>
-          <t>stat_biggest_payout</t>
+          <t>stat_total_paid_out</t>
         </is>
       </c>
       <c r="C703" t="inlineStr">
@@ -21630,12 +21630,12 @@
       </c>
       <c r="D703" t="inlineStr">
         <is>
-          <t>Biggest Payout</t>
+          <t>Total Paid Out</t>
         </is>
       </c>
       <c r="E703" t="inlineStr">
         <is>
-          <t>Mayor Pago</t>
+          <t>Total Pagado</t>
         </is>
       </c>
       <c r="F703" t="b">
@@ -21645,27 +21645,27 @@
     <row r="704">
       <c r="A704" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>Stats</t>
         </is>
       </c>
       <c r="B704" t="inlineStr">
         <is>
-          <t>beecell_statistics_title</t>
+          <t>stat_biggest_payout</t>
         </is>
       </c>
       <c r="C704" t="inlineStr">
         <is>
-          <t>Stats screen title for Beecell</t>
+          <t>Stat row label, Blackjack/Video Poker</t>
         </is>
       </c>
       <c r="D704" t="inlineStr">
         <is>
-          <t>Beecell Statistics</t>
+          <t>Biggest Payout</t>
         </is>
       </c>
       <c r="E704" t="inlineStr">
         <is>
-          <t>Estadísticas de Beecell</t>
+          <t>Mayor Pago</t>
         </is>
       </c>
       <c r="F704" t="b">
@@ -21675,27 +21675,27 @@
     <row r="705">
       <c r="A705" t="inlineStr">
         <is>
-          <t>Casino</t>
+          <t>Shared</t>
         </is>
       </c>
       <c r="B705" t="inlineStr">
         <is>
-          <t>btn_new_bet</t>
+          <t>beecell_statistics_title</t>
         </is>
       </c>
       <c r="C705" t="inlineStr">
         <is>
-          <t>Blackjack action button</t>
+          <t>Stats screen title for Beecell</t>
         </is>
       </c>
       <c r="D705" t="inlineStr">
         <is>
-          <t>New Bet</t>
+          <t>Beecell Statistics</t>
         </is>
       </c>
       <c r="E705" t="inlineStr">
         <is>
-          <t>Nueva Apuesta</t>
+          <t>Estadísticas de Beecell</t>
         </is>
       </c>
       <c r="F705" t="b">
@@ -21710,22 +21710,22 @@
       </c>
       <c r="B706" t="inlineStr">
         <is>
-          <t>btn_rebuy</t>
+          <t>btn_new_bet</t>
         </is>
       </c>
       <c r="C706" t="inlineStr">
         <is>
-          <t>Casino action button to rebuy chips</t>
+          <t>Blackjack action button</t>
         </is>
       </c>
       <c r="D706" t="inlineStr">
         <is>
-          <t>Rebuy</t>
+          <t>New Bet</t>
         </is>
       </c>
       <c r="E706" t="inlineStr">
         <is>
-          <t>Recomprar</t>
+          <t>Nueva Apuesta</t>
         </is>
       </c>
       <c r="F706" t="b">
@@ -21740,25 +21740,55 @@
       </c>
       <c r="B707" t="inlineStr">
         <is>
+          <t>btn_rebuy</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>Casino action button to rebuy chips</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>Rebuy</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>Recomprar</t>
+        </is>
+      </c>
+      <c r="F707" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>Casino</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
           <t>btn_re_deal</t>
         </is>
       </c>
-      <c r="C707" t="inlineStr">
+      <c r="C708" t="inlineStr">
         <is>
           <t>Blackjack action button to deal again</t>
         </is>
       </c>
-      <c r="D707" t="inlineStr">
+      <c r="D708" t="inlineStr">
         <is>
           <t>Re-Deal</t>
         </is>
       </c>
-      <c r="E707" t="inlineStr">
+      <c r="E708" t="inlineStr">
         <is>
           <t>Repartir</t>
         </is>
       </c>
-      <c r="F707" t="b">
+      <c r="F708" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Android: localize the ~45 hard-coded English UI strings
Mac/iOS/Windows route all visible text through the xlsx localization tables,
but Android's Themes, Custom Art Import, About and Manage Decks screens, the
solitaire "New" buttons, Done buttons, the Video Poker pay-table title, the
Blackjack title, the Spider empty-column warning and the Honeycomb Sudden
Death overlay were hard-coded English — Spanish players saw them untranslated.

Reuses existing keys wherever Mac already had the same text (Done, Save,
Cancel, Delete, Edit, Themes, Felt Vignette, Version %@, rule name, etc.) and
adds 12 Android-only keys (pay table title, delete/edit dialogs, import-art
labels, color-channel sliders) to Honeycomb_Localization.xlsx, regenerated for
all platforms. New tr()/trf() composable helpers read the current language.
The Sudden Death overlay now says "Swarm to the Death!" like Mac/Windows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F708"/>
+  <dimension ref="A1:F720"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21789,6 +21789,366 @@
         </is>
       </c>
       <c r="F708" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>AndroidChrome</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>pay_table_title</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>Video Poker pay-table panel title (Android)</t>
+        </is>
+      </c>
+      <c r="D709" t="inlineStr">
+        <is>
+          <t>Pay Table</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>Tabla de Pagos</t>
+        </is>
+      </c>
+      <c r="F709" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>AndroidChrome</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>delete_item_confirm_fmt</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>Confirm-delete dialog title; %@ = item name (Android Themes)</t>
+        </is>
+      </c>
+      <c r="D710" t="inlineStr">
+        <is>
+          <t>Delete %@?</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr">
+        <is>
+          <t>¿Eliminar %@?</t>
+        </is>
+      </c>
+      <c r="F710" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>AndroidChrome</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>theme_asset_delete_body</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>Confirm-delete dialog body for a card back/background/face art (Android Themes)</t>
+        </is>
+      </c>
+      <c r="D711" t="inlineStr">
+        <is>
+          <t>Any theme using this will fall back to a default. This can't be undone.</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr">
+        <is>
+          <t>Cualquier tema que use esto volverá a uno predeterminado. Esto no se puede deshacer.</t>
+        </is>
+      </c>
+      <c r="F711" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>AndroidChrome</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>import_art_button</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>Themes screen top-bar button (Android)</t>
+        </is>
+      </c>
+      <c r="D712" t="inlineStr">
+        <is>
+          <t>Import Art</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>Importar Arte</t>
+        </is>
+      </c>
+      <c r="F712" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>AndroidChrome</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>import_custom_art_title</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>Custom art import screen title (Android)</t>
+        </is>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>Import Custom Art</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>Importar Arte Personalizado</t>
+        </is>
+      </c>
+      <c r="F713" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>AndroidChrome</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>art_type_label</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>Custom art import: art-type picker label (Android)</t>
+        </is>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>Art Type</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>Tipo de Arte</t>
+        </is>
+      </c>
+      <c r="F714" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>AndroidChrome</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>enable_custom_colors_toggle</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>Themes: custom card colors toggle (Android)</t>
+        </is>
+      </c>
+      <c r="D715" t="inlineStr">
+        <is>
+          <t>Enable Custom Colors</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr">
+        <is>
+          <t>Activar Colores Personalizados</t>
+        </is>
+      </c>
+      <c r="F715" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>AndroidChrome</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>edit_item_fmt</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>Edit dialog title; %@ = item name (Android)</t>
+        </is>
+      </c>
+      <c r="D716" t="inlineStr">
+        <is>
+          <t>Edit %@</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr">
+        <is>
+          <t>Editar %@</t>
+        </is>
+      </c>
+      <c r="F716" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>AndroidChrome</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>color_channel_red</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>Color editor slider label (Android)</t>
+        </is>
+      </c>
+      <c r="D717" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>Rojo</t>
+        </is>
+      </c>
+      <c r="F717" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>AndroidChrome</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>color_channel_green</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>Color editor slider label (Android)</t>
+        </is>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>Verde</t>
+        </is>
+      </c>
+      <c r="F718" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>AndroidChrome</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>color_channel_blue</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>Color editor slider label (Android)</t>
+        </is>
+      </c>
+      <c r="D719" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr">
+        <is>
+          <t>Azul</t>
+        </is>
+      </c>
+      <c r="F719" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>AndroidChrome</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>color_channel_alpha</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>Color editor opacity slider label (Android)</t>
+        </is>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>Alpha</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>Opacidad</t>
+        </is>
+      </c>
+      <c r="F720" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Honeycomb: confirm before quitting a match in progress (it counts as a loss)
- Mac: Quit Match now asks "Quit this match? It will count as a loss and end
  your win streak." Cmd+N/Cmd+R are disabled mid-match so they can't abandon it
  silently.
- Windows: same confirmation on Quit Match; Ctrl+N/Ctrl+R ignored mid-match.
- iOS/Android already confirmed - now with the same wording (was the generic
  new-match text).
- Two new phrases in the localization sheet, plus Windows' untranslated
  "Discard Changes?" dialog (Options > Cancel with unsaved changes).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F728"/>
+  <dimension ref="A1:F732"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22389,6 +22389,126 @@
         </is>
       </c>
       <c r="F728" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>Honeycomb</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>quit_match_confirm_title</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>Confirm before quitting a Honeycomb match in progress</t>
+        </is>
+      </c>
+      <c r="D729" t="inlineStr">
+        <is>
+          <t>Quit this match?</t>
+        </is>
+      </c>
+      <c r="E729" t="inlineStr">
+        <is>
+          <t>¿Abandonar esta partida?</t>
+        </is>
+      </c>
+      <c r="F729" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>Honeycomb</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>quit_match_confirm_body</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>Body of the quit-match confirmation</t>
+        </is>
+      </c>
+      <c r="D730" t="inlineStr">
+        <is>
+          <t>It will count as a loss and end your win streak.</t>
+        </is>
+      </c>
+      <c r="E730" t="inlineStr">
+        <is>
+          <t>Contará como una derrota y terminará tu racha de victorias.</t>
+        </is>
+      </c>
+      <c r="F730" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>WindowsChrome</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>discard_changes_title</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>Windows Options: cancel with unsaved changes</t>
+        </is>
+      </c>
+      <c r="D731" t="inlineStr">
+        <is>
+          <t>Discard Changes?</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr">
+        <is>
+          <t>¿Descartar cambios?</t>
+        </is>
+      </c>
+      <c r="F731" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>WindowsChrome</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>discard_changes_body</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>Windows Options: cancel with unsaved changes</t>
+        </is>
+      </c>
+      <c r="D732" t="inlineStr">
+        <is>
+          <t>You have pending changes which will be lost. Are you sure you want to cancel?</t>
+        </is>
+      </c>
+      <c r="E732" t="inlineStr">
+        <is>
+          <t>Tienes cambios pendientes que se perderán. ¿Seguro que quieres cancelar?</t>
+        </is>
+      </c>
+      <c r="F732" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
iOS App Store prep: privacy manifest, export compliance, no betting language
- PrivacyInfo.xcprivacy: no tracking, no data collected; declares the one
  required-reason API the app uses (UserDefaults, CA92.1) so uploads aren't
  flagged.
- ITSAppUsesNonExemptEncryption = NO, so App Store Connect stops asking the
  export-compliance question on every upload.
- Betting is locked off on iOS, but the Video Poker and Blackjack help pages
  still described bets, coins, the 800x jackpot and payouts, the game picker
  called Video Poker "casino poker with pay tables", and both stats screens
  listed Total Wagered / Total Paid / Return to Player / Biggest Payout /
  Rebuys (always 0). iOS now gets betting-free help text (6 new phrases,
  English + Spanish) and stats without the money rows. Mac/Windows/Android
  unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F732"/>
+  <dimension ref="A1:F738"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22509,6 +22509,220 @@
         </is>
       </c>
       <c r="F732" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>HelpIOS</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>help_videopoker_subtitle_ios</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>iOS help/game picker — betting is locked off on iOS (App Store), so no bets, coins, credits, payouts or jackpots</t>
+        </is>
+      </c>
+      <c r="D733" t="inlineStr">
+        <is>
+          <t>Classic draw poker with Jacks or Better, Deuces Wild, and Bonus Poker variants.</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr">
+        <is>
+          <t>Póker de descarte clásico con las variantes Jacks or Better, Deuces Wild y Bonus Poker.</t>
+        </is>
+      </c>
+      <c r="F733" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>HelpIOS</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>help_videopoker_objective_ios</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>iOS help/game picker — betting is locked off on iOS (App Store), so no bets, coins, credits, payouts or jackpots</t>
+        </is>
+      </c>
+      <c r="D734" t="inlineStr">
+        <is>
+          <t>Draw the best 5-card poker hand you can. Each variant has its own lowest winning hand.</t>
+        </is>
+      </c>
+      <c r="E734" t="inlineStr">
+        <is>
+          <t>Consigue la mejor mano de póker de 5 cartas posible. Cada variante tiene su propia mano ganadora mínima.</t>
+        </is>
+      </c>
+      <c r="F734" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>HelpIOS</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>help_videopoker_how_to_play_ios</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>iOS help/game picker — betting is locked off on iOS (App Store), so no bets, coins, credits, payouts or jackpots</t>
+        </is>
+      </c>
+      <c r="D735" t="inlineStr">
+        <is>
+          <t>1. Deal: Tap Deal to receive 5 cards.
+2. Hold: Tap the cards you want to keep.
+3. Draw: Tap Draw. Unheld cards are replaced and your final hand is scored.
+Game Variants:
+• Jacks or Better: The lowest winning hand is a pair of Jacks, Queens, Kings, or Aces.
+• Deuces Wild: All four 2s are wild cards. The lowest winning hand is Three of a Kind.
+• Bonus Poker: Like Jacks or Better, with extra emphasis on Four of a Kind (Four Aces and Four 2s–4s stand out).</t>
+        </is>
+      </c>
+      <c r="E735" t="inlineStr">
+        <is>
+          <t>1. Repartir: Toca Repartir para recibir 5 cartas.
+2. Retener: Toca las cartas que quieras conservar.
+3. Robar: Toca Robar. Las cartas no retenidas se reemplazan y se puntúa tu mano final.
+Variantes:
+• Jacks or Better: La mano ganadora mínima es un par de Jotas, Reinas, Reyes o Ases.
+• Deuces Wild: Los cuatro 2 son comodines. La mano ganadora mínima es un Trío.
+• Bonus Poker: Como Jacks or Better, con especial énfasis en el Póker (destacan Cuatro Ases y Cuatro 2–4).</t>
+        </is>
+      </c>
+      <c r="F735" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>HelpIOS</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>help_videopoker_strategy_ios</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>iOS help/game picker — betting is locked off on iOS (App Store), so no bets, coins, credits, payouts or jackpots</t>
+        </is>
+      </c>
+      <c r="D736" t="inlineStr">
+        <is>
+          <t>1. Never Break a Made Hand (Except for 4-to-a-Royal): Only break a Straight or Flush if you are 1 card away from a Royal Flush.
+2. In Deuces Wild, Never Discard a 2: Deuces are wild—always hold every 2 dealt to you!
+3. Nothing Dealt? Hold your high cards (Jack or better) to chase a winning pair.</t>
+        </is>
+      </c>
+      <c r="E736" t="inlineStr">
+        <is>
+          <t>1. Nunca rompas una mano hecha (salvo 4 cartas de Escalera Real): Solo rompe una Escalera o un Color si te falta 1 carta para una Escalera Real.
+2. En Deuces Wild, nunca descartes un 2: ¡Los doses son comodines, retén siempre cada 2!
+3. ¿Sin nada? Retén tus cartas altas (Jota o más) para buscar un par ganador.</t>
+        </is>
+      </c>
+      <c r="F736" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>HelpIOS</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>help_blackjack_rules_ios</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>iOS help/game picker — betting is locked off on iOS (App Store), so no bets, coins, credits, payouts or jackpots</t>
+        </is>
+      </c>
+      <c r="D737" t="inlineStr">
+        <is>
+          <t>1. Deal: Tap Deal to start a hand.
+2. Your Turn:
+  – Hit: Take another card.
+  – Stand: Keep your current hand.
+  – Double Down: Take exactly 1 more card and automatically stand. (Available on initial 2 cards with totals of 9, 10, or 11).
+  – Split: If dealt two matching ranks, play them as two separate hands.
+3. Dealer's Turn: Dealer reveals their hidden card and must hit until reaching 17 or higher (stands on all 17s).
+Results: Finish closer to 21 than the dealer without going over to win the hand. A tie is a push.</t>
+        </is>
+      </c>
+      <c r="E737" t="inlineStr">
+        <is>
+          <t>1. Repartir: Toca Repartir para empezar una mano.
+2. Tu turno:
+  – Pedir: Toma otra carta.
+  – Plantarse: Conserva tu mano actual.
+  – Doblar: Toma exactamente 1 carta más y plántate automáticamente. (Disponible con las 2 cartas iniciales si suman 9, 10 u 11).
+  – Dividir: Si recibes dos cartas del mismo rango, juégalas como dos manos separadas.
+3. Turno del crupier: El crupier revela su carta oculta y debe pedir hasta llegar a 17 o más (se planta con cualquier 17).
+Resultados: Termina más cerca de 21 que el crupier sin pasarte para ganar la mano. Un empate es un push.</t>
+        </is>
+      </c>
+      <c r="F737" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>HelpIOS</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>help_blackjack_strategy_ios</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>iOS help/game picker — betting is locked off on iOS (App Store), so no bets, coins, credits, payouts or jackpots</t>
+        </is>
+      </c>
+      <c r="D738" t="inlineStr">
+        <is>
+          <t>1. Always Split Aces and 8s: Never split 10s or 5s.
+2. Double Down on 11: Always Double Down when your starting hand totals 11 against a dealer 2 through 10.
+3. Watch the Dealer's Upcard: If the dealer shows a 2 through 6, they have a high chance of busting—stand on hard 12 or higher and let the dealer draw.</t>
+        </is>
+      </c>
+      <c r="E738" t="inlineStr">
+        <is>
+          <t>1. Divide siempre Ases y 8: Nunca dividas 10 ni 5.
+2. Dobla con 11: Dobla siempre cuando tu mano inicial sume 11 contra un 2 a 10 del crupier.
+3. Observa la carta visible del crupier: Si muestra de 2 a 6, tiene muchas probabilidades de pasarse; plántate con 12 duro o más y deja que el crupier pida.</t>
+        </is>
+      </c>
+      <c r="F738" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Android: remove betting to match iOS
- Video Poker and Blackjack are hard-locked to free play (isFreePlay always
  true), so bet controls, credits, payouts, Rebuy and the out-of-credits toast
  are all off; the Credits/Bet/Hands panel and the pay table it opened are gone.
- Options: no Starting Credits / Default Bet; Blackjack's only setting was
  Starting Credits, so it has no game section now. Help is the betting-free guide
  iOS uses.
- Stats: no money rows (wagered, paid, biggest payout, return to player, rebuys).
- Klondike: Vegas scoring locked off (toggle removed; a previously saved Vegas
  setting is ignored); help shows the rules without Vegas.
- Game picker: betting-free Video Poker description, and a Klondike one-liner
  without "Vegas scoring" - now also used on iOS, whose picker and help still
  advertised Vegas scoring it doesn't have (new phrase, English + Spanish).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F739"/>
+  <dimension ref="A1:F740"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22767,6 +22767,36 @@
         </is>
       </c>
       <c r="F739" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>HelpIOS</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>help_klondike_subtitle_ios</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>Klondike one-liner on mobile (iOS/Android) — no Vegas scoring there</t>
+        </is>
+      </c>
+      <c r="D740" t="inlineStr">
+        <is>
+          <t>Classic single-deck solitaire with Draw 1 and Draw 3 modes.</t>
+        </is>
+      </c>
+      <c r="E740" t="inlineStr">
+        <is>
+          <t>Clásico solitario de un mazo con modos Robar 1 y Robar 3.</t>
+        </is>
+      </c>
+      <c r="F740" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
App Store hardening: remove Android Blackjack New Bet button, rename Video Poker to Draw Poker, drop 'Get rich' idle line, square iOS app icon
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -4562,12 +4562,12 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Video Poker Help</t>
+          <t>Draw Poker Help</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Ayuda de Video Póker</t>
+          <t>Ayuda de Póker de Descarte</t>
         </is>
       </c>
       <c r="F138" t="b">
@@ -10564,12 +10564,12 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Video Poker Statistics</t>
+          <t>Draw Poker Statistics</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>Estadísticas de Video Póker</t>
+          <t>Estadísticas de Póker de Descarte</t>
         </is>
       </c>
       <c r="F338" t="b">
@@ -15420,12 +15420,12 @@
       </c>
       <c r="D496" t="inlineStr">
         <is>
-          <t>Video Poker</t>
+          <t>Draw Poker</t>
         </is>
       </c>
       <c r="E496" t="inlineStr">
         <is>
-          <t>Video Póker</t>
+          <t>Póker de Descarte</t>
         </is>
       </c>
       <c r="F496" t="b">
@@ -17610,12 +17610,12 @@
       </c>
       <c r="D569" t="inlineStr">
         <is>
-          <t>VIDEO POKER</t>
+          <t>DRAW POKER</t>
         </is>
       </c>
       <c r="E569" t="inlineStr">
         <is>
-          <t>VIDEO POKER</t>
+          <t>PÓKER DE DESCARTE</t>
         </is>
       </c>
       <c r="F569" t="b">
@@ -22991,7 +22991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F288"/>
+  <dimension ref="A1:F287"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31519,7 +31519,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Get rich or buzz trying.</t>
+          <t>To bee, or not to bee... wait, whose turn is it?</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
@@ -31551,7 +31551,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>To bee, or not to bee... wait, whose turn is it?</t>
+          <t>May the swarm be with you.</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
@@ -31566,7 +31566,7 @@
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>No Translation</t>
+          <t>Que el enjambre te acompañe.</t>
         </is>
       </c>
     </row>
@@ -31583,7 +31583,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>May the swarm be with you.</t>
+          <t>Live, Laugh, Pollinate.</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
@@ -31598,7 +31598,7 @@
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>Que el enjambre te acompañe.</t>
+          <t>Vive, Ríe, Poliniza.</t>
         </is>
       </c>
     </row>
@@ -31615,7 +31615,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Live, Laugh, Pollinate.</t>
+          <t>Keep calm and buzz on.</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
@@ -31630,7 +31630,7 @@
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>Vive, Ríe, Poliniza.</t>
+          <t>No Translation</t>
         </is>
       </c>
     </row>
@@ -31647,7 +31647,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Keep calm and buzz on.</t>
+          <t>Home is where the hive is.</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
@@ -31662,7 +31662,7 @@
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>No Translation</t>
+          <t>El hogar está donde está la colmena.</t>
         </is>
       </c>
     </row>
@@ -31679,7 +31679,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Home is where the hive is.</t>
+          <t>Just a worker bee looking for my queen.</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
@@ -31694,7 +31694,7 @@
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>El hogar está donde está la colmena.</t>
+          <t>Solo una abeja obrera buscando a mi reina.</t>
         </is>
       </c>
     </row>
@@ -31711,7 +31711,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Just a worker bee looking for my queen.</t>
+          <t>Are you gonna play a card, or just sit there looking sweet?</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
@@ -31726,7 +31726,7 @@
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>Solo una abeja obrera buscando a mi reina.</t>
+          <t>¿Vas a jugar una carta, o solo te vas a sentar ahí luciendo dulce?</t>
         </is>
       </c>
     </row>
@@ -31743,7 +31743,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Are you gonna play a card, or just sit there looking sweet?</t>
+          <t>Frankly, my dear, I don't give a buzz.</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
@@ -31758,7 +31758,7 @@
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>¿Vas a jugar una carta, o solo te vas a sentar ahí luciendo dulce?</t>
+          <t>No Translation</t>
         </is>
       </c>
     </row>
@@ -31775,7 +31775,7 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Frankly, my dear, I don't give a buzz.</t>
+          <t>We're gonna need a bigger hive.</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
@@ -31790,7 +31790,7 @@
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>No Translation</t>
+          <t>Vamos a necesitar una colmena más grande.</t>
         </is>
       </c>
     </row>
@@ -31807,7 +31807,7 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>We're gonna need a bigger hive.</t>
+          <t>Show me the honey!</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
@@ -31822,7 +31822,7 @@
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>Vamos a necesitar una colmena más grande.</t>
+          <t>¡Muéstrame la miel!</t>
         </is>
       </c>
     </row>
@@ -31839,7 +31839,7 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Show me the honey!</t>
+          <t>I'll bee back.</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
@@ -31854,7 +31854,7 @@
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>¡Muéstrame la miel!</t>
+          <t>No Translation</t>
         </is>
       </c>
     </row>
@@ -31871,7 +31871,7 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>I'll bee back.</t>
+          <t>Nobody puts Baby Bee in a corner.</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
@@ -31886,7 +31886,7 @@
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>No Translation</t>
+          <t>Nadie pone a Abeja Bebé en un rincón.</t>
         </is>
       </c>
     </row>
@@ -31903,7 +31903,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Nobody puts Baby Bee in a corner.</t>
+          <t>Sweet dreams are made of bees.</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
@@ -31918,7 +31918,7 @@
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>Nadie pone a Abeja Bebé en un rincón.</t>
+          <t>No Translation</t>
         </is>
       </c>
     </row>
@@ -31935,7 +31935,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Sweet dreams are made of bees.</t>
+          <t>Bee yourself; everyone else is already taken.</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
@@ -31967,7 +31967,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Bee yourself; everyone else is already taken.</t>
+          <t>Mind your own beeswax!</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
@@ -31999,7 +31999,7 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Mind your own beeswax!</t>
+          <t>This one weird trick captures 4 cards at once — dealers don't want you to know it.</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
@@ -32014,7 +32014,7 @@
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>No Translation</t>
+          <t>Este extraño truco captura 4 cartas a la vez — los repartidores no quieren que lo sepas.</t>
         </is>
       </c>
     </row>
@@ -32031,7 +32031,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>This one weird trick captures 4 cards at once — dealers don't want you to know it.</t>
+          <t>You won't believe what happened when a worker bee met a Fallen Ace.</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -32046,7 +32046,7 @@
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>Este extraño truco captura 4 cartas a la vez — los repartidores no quieren que lo sepas.</t>
+          <t>No vas a creer lo que pasó cuando una abeja obrera conoció a un As Caído.</t>
         </is>
       </c>
     </row>
@@ -32063,7 +32063,7 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>You won't believe what happened when a worker bee met a Fallen Ace.</t>
+          <t>She said yes to Symmetry. He said yes to Math Bee. Chaos ensued.</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -32078,29 +32078,29 @@
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>No vas a creer lo que pasó cuando una abeja obrera conoció a un As Caído.</t>
+          <t>Ella dijo sí a la Simetría. Él dijo sí a Abeja Matemática. Se desató el caos.</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>Idle Action</t>
+          <t>Gameplay</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>No action taken for one minute.</t>
+          <t>Player runs out of credits (Video Poker/Blackjack).</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>She said yes to Symmetry. He said yes to Math Bee. Chaos ensued.</t>
+          <t>Busy as a bee, broke as a beekeeper.</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Ambiance</t>
+          <t>Repeatable Flavor</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -32110,29 +32110,29 @@
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>Ella dijo sí a la Simetría. Él dijo sí a Abeja Matemática. Se desató el caos.</t>
+          <t>Ocupado como una abeja, arruinado como un apicultor.</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>Gameplay</t>
+          <t>Idle Action</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Player runs out of credits (Video Poker/Blackjack).</t>
+          <t>No action taken for one minute.</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Busy as a bee, broke as a beekeeper.</t>
+          <t>Absence makes the heart grow fonder — and the hive grow louder.</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Repeatable Flavor</t>
+          <t>Ambiance</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -32142,7 +32142,7 @@
       </c>
       <c r="F286" t="inlineStr">
         <is>
-          <t>Ocupado como una abeja, arruinado como un apicultor.</t>
+          <t>La ausencia hace que el corazón se encariñe — y la colmena suene más fuerte.</t>
         </is>
       </c>
     </row>
@@ -32159,7 +32159,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>Absence makes the heart grow fonder — and the hive grow louder.</t>
+          <t>Two bees or not two bees — that's a math problem, not a question.</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
@@ -32173,38 +32173,6 @@
         </is>
       </c>
       <c r="F287" t="inlineStr">
-        <is>
-          <t>La ausencia hace que el corazón se encariñe — y la colmena suene más fuerte.</t>
-        </is>
-      </c>
-    </row>
-    <row r="288">
-      <c r="A288" t="inlineStr">
-        <is>
-          <t>Idle Action</t>
-        </is>
-      </c>
-      <c r="B288" t="inlineStr">
-        <is>
-          <t>No action taken for one minute.</t>
-        </is>
-      </c>
-      <c r="C288" t="inlineStr">
-        <is>
-          <t>Two bees or not two bees — that's a math problem, not a question.</t>
-        </is>
-      </c>
-      <c r="D288" t="inlineStr">
-        <is>
-          <t>Ambiance</t>
-        </is>
-      </c>
-      <c r="E288" t="inlineStr">
-        <is>
-          <t>Toast</t>
-        </is>
-      </c>
-      <c r="F288" t="inlineStr">
         <is>
           <t>No Translation</t>
         </is>

</xml_diff>

<commit_message>
Rule text: Sudden Death reads the same everywhere; Scouting Party fallback matches Mac
Sudden Death now says the cards each player currently owns become their new hand and the match
restarts immediately (spreadsheet, so Mac/iOS, Windows and Android all show it; English and Spanish),
including the built-in fallbacks. Windows' unused Scouting Party fallback now matches the
spreadsheet text Mac shows. Tests check the wording.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -17040,12 +17040,12 @@
       </c>
       <c r="D550" t="inlineStr">
         <is>
-          <t>If the match ends in a draw, a rematch begins immediately.</t>
+          <t>If the match ends in a draw, the cards currently owned by each player become their new hand and the match restarts immediately.</t>
         </is>
       </c>
       <c r="E550" t="inlineStr">
         <is>
-          <t>Si la partida termina en empate, comienza una revancha inmediatamente.</t>
+          <t>Si la partida termina en empate, las cartas que posee cada jugador en ese momento se convierten en su nueva mano y la partida se reinicia de inmediato.</t>
         </is>
       </c>
       <c r="F550" t="b">

</xml_diff>